<commit_message>
report: add Karnaugh map groupings
</commit_message>
<xml_diff>
--- a/deliverables/Карты_Карно_Блинов.xlsx
+++ b/deliverables/Карты_Карно_Блинов.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переходы" sheetId="1" r:id="R82a1e5d52c4f418e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Карты Карно" sheetId="2" r:id="R80e440adcfc14a3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Переходы" sheetId="1" r:id="R9ea95d29357b43d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Карты Карно" sheetId="2" r:id="R7d2e635721b74062"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -338,7 +338,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -349,7 +349,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -360,7 +360,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFEB9C"/>
         </x:patternFill>
       </x:fill>
@@ -371,7 +371,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -382,7 +382,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -393,7 +393,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFEB9C"/>
         </x:patternFill>
       </x:fill>
@@ -404,7 +404,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -415,7 +415,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -426,7 +426,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFEB9C"/>
         </x:patternFill>
       </x:fill>
@@ -437,7 +437,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -448,7 +448,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFC7CE"/>
         </x:patternFill>
       </x:fill>
@@ -459,13 +459,732 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFEB9C"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
   </x:dxfs>
 </x:styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2362200" cy="238125"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1" name="KMap_D3_G1"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="2362200" cy="238125"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="006BB6"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1143000" cy="552450"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="KMap_D3_G2"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="1143000" cy="552450"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="38A800"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="514350" cy="219075"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="KMap_D3_G3_L"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="514350" cy="219075"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="E31A1C"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="514350" cy="219075"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="KMap_D3_G3_R"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="514350" cy="219075"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="E31A1C"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="533400" cy="552450"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="KMap_D2_G1"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="533400" cy="552450"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="E31A1C"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="533400" cy="552450"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="KMap_D2_G2"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="533400" cy="552450"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="38A800"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1143000" cy="238125"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="KMap_D2_G3_T"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="1143000" cy="238125"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="006BB6"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1143000" cy="238125"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="KMap_D2_G3_B"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="1143000" cy="238125"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="006BB6"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="457200" cy="161925"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="KMap_D2_G4_TL"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="457200" cy="161925"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="8E44AD"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="457200" cy="161925"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="KMap_D2_G4_TR"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="457200" cy="161925"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="8E44AD"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="457200" cy="161925"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="KMap_D2_G4_BL"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="457200" cy="161925"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="8E44AD"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="457200" cy="161925"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="12" name="KMap_D2_G4_BR"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="457200" cy="161925"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="8E44AD"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1143000" cy="238125"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="13" name="KMap_D1_G1"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="1143000" cy="238125"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="006BB6"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1143000" cy="238125"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="14" name="KMap_D1_G2"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="1143000" cy="238125"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="38A800"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1143000" cy="238125"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="15" name="KMap_D1_G3"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="1143000" cy="238125"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="8E44AD"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="533400" cy="552450"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="16" name="KMap_D1_G4"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="533400" cy="552450"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="E31A1C"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1143000" cy="238125"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="17" name="KMap_D0_G1"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="1143000" cy="238125"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="38A800"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="514350" cy="219075"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="18" name="KMap_D0_G2_T"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="514350" cy="219075"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="E31A1C"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="514350" cy="219075"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="19" name="KMap_D0_G2_B"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="514350" cy="219075"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="E31A1C"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="533400" cy="552450"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="20" name="KMap_D0_G3_L"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="533400" cy="552450"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="006BB6"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="533400" cy="552450"/>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="21" name="KMap_D0_G3_R"/>
+        <xdr:cNvSpPr>
+          <a:spLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noGrp="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="0" y="0"/>
+          <a:ext cx="533400" cy="552450"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="21431">
+          <a:solidFill>
+            <a:srgbClr val="006BB6"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2011,37 +2730,37 @@
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
       <x:c r="A19" s="52" t="str">
-        <x:v>1 — единичный набор; 0 — нулевой набор; X — неиспользуемое состояние</x:v>
+        <x:v>Овалы одного цвета — одна группа; парные овалы у границ — склейка через край; X — факультативный набор</x:v>
       </x:c>
       <x:c r="B19" s="53" t="str">
-        <x:v>1 — единичный набор; 0 — нулевой набор; X — неиспользуемое состояние</x:v>
+        <x:v>Овалы одного цвета — одна группа; парные овалы у границ — склейка через край; X — факультативный набор</x:v>
       </x:c>
       <x:c r="C19" s="53" t="str">
-        <x:v>1 — единичный набор; 0 — нулевой набор; X — неиспользуемое состояние</x:v>
+        <x:v>Овалы одного цвета — одна группа; парные овалы у границ — склейка через край; X — факультативный набор</x:v>
       </x:c>
       <x:c r="D19" s="53" t="str">
-        <x:v>1 — единичный набор; 0 — нулевой набор; X — неиспользуемое состояние</x:v>
+        <x:v>Овалы одного цвета — одна группа; парные овалы у границ — склейка через край; X — факультативный набор</x:v>
       </x:c>
       <x:c r="E19" s="53" t="str">
-        <x:v>1 — единичный набор; 0 — нулевой набор; X — неиспользуемое состояние</x:v>
+        <x:v>Овалы одного цвета — одна группа; парные овалы у границ — склейка через край; X — факультативный набор</x:v>
       </x:c>
       <x:c r="F19" s="53" t="str">
-        <x:v>1 — единичный набор; 0 — нулевой набор; X — неиспользуемое состояние</x:v>
+        <x:v>Овалы одного цвета — одна группа; парные овалы у границ — склейка через край; X — факультативный набор</x:v>
       </x:c>
       <x:c r="G19" s="53" t="str">
-        <x:v>1 — единичный набор; 0 — нулевой набор; X — неиспользуемое состояние</x:v>
+        <x:v>Овалы одного цвета — одна группа; парные овалы у границ — склейка через край; X — факультативный набор</x:v>
       </x:c>
       <x:c r="H19" s="53" t="str">
-        <x:v>1 — единичный набор; 0 — нулевой набор; X — неиспользуемое состояние</x:v>
+        <x:v>Овалы одного цвета — одна группа; парные овалы у границ — склейка через край; X — факультативный набор</x:v>
       </x:c>
       <x:c r="I19" s="53" t="str">
-        <x:v>1 — единичный набор; 0 — нулевой набор; X — неиспользуемое состояние</x:v>
+        <x:v>Овалы одного цвета — одна группа; парные овалы у границ — склейка через край; X — факультативный набор</x:v>
       </x:c>
       <x:c r="J19" s="53" t="str">
-        <x:v>1 — единичный набор; 0 — нулевой набор; X — неиспользуемое состояние</x:v>
+        <x:v>Овалы одного цвета — одна группа; парные овалы у границ — склейка через край; X — факультативный набор</x:v>
       </x:c>
       <x:c r="K19" s="54" t="str">
-        <x:v>1 — единичный набор; 0 — нулевой набор; X — неиспользуемое состояние</x:v>
+        <x:v>Овалы одного цвета — одна группа; парные овалы у границ — склейка через край; X — факультативный набор</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2094,5 +2813,6 @@
     <x:cfRule type="containsText" dxfId="11" priority="12" operator="containsText" text="X"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d2d272eb9e747ce"/>
 </x:worksheet>
 </file>
</xml_diff>